<commit_message>
model: add fodder (oil-cake) margin sheet — Rs15.5cr/17% of revenue; without it oil-only EBITDA is -Rs2.7cr (fodder makes the mill viable); TN Namakkal poultry + Aavin dairy demand; updated TN cake prices
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pitch/TN-Combined-Oil-Mill-Model.xlsx
+++ b/pitch/TN-Combined-Oil-Mill-Model.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per-Line Economics" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Combined P&amp;L &amp; Returns" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coconut-Price Sensitivity" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEA Prices &amp; Sources" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fodder (Oil-Cake) Margin" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEA Prices &amp; Sources" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -124,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,6 +155,8 @@
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -652,7 +655,7 @@
         <v>175000</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>27000</v>
+        <v>32000</v>
       </c>
     </row>
     <row r="9">
@@ -679,7 +682,7 @@
         <v>250000</v>
       </c>
       <c r="H9" s="6" t="n">
-        <v>35000</v>
+        <v>42000</v>
       </c>
     </row>
     <row r="11">
@@ -893,7 +896,7 @@
         </is>
       </c>
       <c r="C7" s="11" t="n">
-        <v>23.4</v>
+        <v>24.0875</v>
       </c>
       <c r="D7" s="11" t="n">
         <v>22.5</v>
@@ -902,16 +905,16 @@
         <v>1.75</v>
       </c>
       <c r="F7" s="11" t="n">
-        <v>-0.8500000000000014</v>
+        <v>-0.1625000000000014</v>
       </c>
       <c r="G7" s="12" t="n">
-        <v>-0.03632478632478639</v>
+        <v>-0.006746237675142768</v>
       </c>
       <c r="H7" s="15" t="n">
-        <v>-0.8500000000000014</v>
+        <v>-0.1625000000000014</v>
       </c>
       <c r="I7" s="16" t="n">
-        <v>-0.03632478632478639</v>
+        <v>-0.006746237675142768</v>
       </c>
     </row>
     <row r="8">
@@ -921,7 +924,7 @@
         </is>
       </c>
       <c r="C8" s="11" t="n">
-        <v>51.135</v>
+        <v>51.912</v>
       </c>
       <c r="D8" s="11" t="n">
         <v>36</v>
@@ -930,16 +933,16 @@
         <v>2.1</v>
       </c>
       <c r="F8" s="11" t="n">
-        <v>13.035</v>
+        <v>13.812</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>0.2549134643590495</v>
+        <v>0.2660656495607952</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>13.035</v>
+        <v>13.812</v>
       </c>
       <c r="I8" s="14" t="n">
-        <v>0.2549134643590495</v>
+        <v>0.2660656495607952</v>
       </c>
     </row>
     <row r="9">
@@ -949,7 +952,7 @@
         </is>
       </c>
       <c r="C9" s="18" t="n">
-        <v>92.229</v>
+        <v>93.6935</v>
       </c>
       <c r="D9" s="18" t="n">
         <v>70.5</v>
@@ -958,7 +961,7 @@
         <v>8.050000000000001</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>13.679</v>
+        <v>15.1435</v>
       </c>
     </row>
     <row r="11">
@@ -1043,7 +1046,7 @@
         </is>
       </c>
       <c r="C6" s="18" t="n">
-        <v>92.229</v>
+        <v>93.6935</v>
       </c>
     </row>
     <row r="7">
@@ -1073,7 +1076,7 @@
         </is>
       </c>
       <c r="C9" s="11" t="n">
-        <v>2.76687</v>
+        <v>2.810805</v>
       </c>
     </row>
     <row r="10">
@@ -1083,7 +1086,7 @@
         </is>
       </c>
       <c r="C10" s="18" t="n">
-        <v>10.91213</v>
+        <v>12.332695</v>
       </c>
     </row>
     <row r="11">
@@ -1093,7 +1096,7 @@
         </is>
       </c>
       <c r="C11" s="12" t="n">
-        <v>0.1183156057205434</v>
+        <v>0.1316280745195771</v>
       </c>
     </row>
     <row r="12">
@@ -1113,7 +1116,7 @@
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>9.912129999999998</v>
+        <v>11.332695</v>
       </c>
     </row>
     <row r="14">
@@ -1133,7 +1136,7 @@
         </is>
       </c>
       <c r="C15" s="11" t="n">
-        <v>7.864629999999998</v>
+        <v>9.285195</v>
       </c>
     </row>
     <row r="16">
@@ -1143,7 +1146,7 @@
         </is>
       </c>
       <c r="C16" s="11" t="n">
-        <v>1.9661575</v>
+        <v>2.32129875</v>
       </c>
     </row>
     <row r="17">
@@ -1153,7 +1156,7 @@
         </is>
       </c>
       <c r="C17" s="18" t="n">
-        <v>5.898472499999999</v>
+        <v>6.963896249999999</v>
       </c>
     </row>
     <row r="18">
@@ -1163,7 +1166,7 @@
         </is>
       </c>
       <c r="C18" s="12" t="n">
-        <v>0.06395464008066876</v>
+        <v>0.07432635401602032</v>
       </c>
     </row>
     <row r="20">
@@ -1188,7 +1191,7 @@
         </is>
       </c>
       <c r="C21" s="23" t="n">
-        <v>0.3705992929560952</v>
+        <v>0.4118458698259618</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1203,7 +1206,7 @@
         </is>
       </c>
       <c r="C22" s="24" t="n">
-        <v>0.3964851999999999</v>
+        <v>0.4533078</v>
       </c>
     </row>
     <row r="23">
@@ -1213,7 +1216,7 @@
         </is>
       </c>
       <c r="C23" s="25" t="n">
-        <v>3.325198858356564</v>
+        <v>3.721214589141112</v>
       </c>
     </row>
     <row r="24">
@@ -1223,11 +1226,11 @@
         </is>
       </c>
       <c r="C24" s="24" t="n">
-        <v>0.1183156057205434</v>
+        <v>0.1316280745195771</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>PAT 6.4%</t>
+          <t>PAT 7.4%</t>
         </is>
       </c>
     </row>
@@ -1300,19 +1303,19 @@
         </is>
       </c>
       <c r="C7" s="26" t="n">
-        <v>1.462129999999999</v>
+        <v>2.882695000000001</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>6.187129999999994</v>
+        <v>7.607694999999994</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>10.91212999999999</v>
+        <v>12.332695</v>
       </c>
       <c r="F7" s="28" t="n">
-        <v>15.63713</v>
+        <v>17.057695</v>
       </c>
       <c r="G7" s="28" t="n">
-        <v>20.36213</v>
+        <v>21.782695</v>
       </c>
     </row>
     <row r="9">
@@ -1363,6 +1366,290 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:J25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Fodder margin — the oil cake that makes the mill viable</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Oil cakes sold as cattle/poultry feed = 17% of revenue and the STABLE base. Without it, oil-only EBITDA is negative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Oil cake (fodder)</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>From line</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Volume t/yr</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Feed ₹/kg</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Protein</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Revenue ₹cr</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>TN buyer</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DORB (de-oiled rice bran)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Rice bran</t>
+        </is>
+      </c>
+      <c r="D6" s="29" t="n">
+        <v>4980</v>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>13</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>~15%</t>
+        </is>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>6.474</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Aavin dairy / aqua feed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Groundnut cake / DOC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Groundnut</t>
+        </is>
+      </c>
+      <c r="D7" s="29" t="n">
+        <v>1375</v>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>40-50%</t>
+        </is>
+      </c>
+      <c r="G7" s="11" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Namakkal poultry (premium protein)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Coconut oil cake (poonac)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Copra</t>
+        </is>
+      </c>
+      <c r="D8" s="29" t="n">
+        <v>1110</v>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>42</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>~20%</t>
+        </is>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>4.662</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Aavin cattle / Kangayam cattle</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>TOTAL FODDER REVENUE</t>
+        </is>
+      </c>
+      <c r="G9" s="30" t="n">
+        <v>15.536</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>WHY FODDER IS ESSENTIAL, NOT INCREMENTAL</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+      <c r="I11" s="4" t="n"/>
+      <c r="J11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>Oil revenue only:                 ₹78.2 cr</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>+ Fodder (oil-cake) revenue:      ₹15.5 cr (17%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="20">
+        <f> Total revenue:                  ₹93.7 cr</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="20" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>→ EBITDA with fodder:   +₹12.3 cr (13.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>→ EBITDA WITHOUT fodder: about -₹3 cr (LOSS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>The oil cake is the difference between a loss-making and a profitable mill — the classic crush-margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>reality (oil + meal - seed). It also makes the groundnut line viable (better cake price lifts it from -4% to -1%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>→ STABLE base: feed prices do NOT swing like coconut oil (which moved 2x in 2025). Fodder is the</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  de-risker against oil-price volatility — steady ₹15.5 cr floor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="19" t="inlineStr">
+        <is>
+          <t>→ CAPTIVE local demand: Namakkal (India's #2 egg centre, 80% of TN layer farms) + Aavin dairy</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  (Erode cattle-feed plant 150 MT/day, offtake up 20x in 8 yrs) are IN the oil belt — minimal logistics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="19" t="inlineStr">
+        <is>
+          <t>→ Groundnut cake (40-50% protein) commands the premium; DORB and coconut cake are volume feed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1391,166 +1678,166 @@
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="29" t="inlineStr">
+      <c r="B5" s="31" t="inlineStr">
         <is>
           <t>FEEDSTOCK &amp; OIL PRICES (₹/tonne, TN/SEA/market 2026)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="29" t="inlineStr">
+      <c r="B6" s="31" t="inlineStr">
         <is>
           <t>• Rice bran ₹20,000 (Coimbatore); Refined RBO ₹110,000 (SEA daily rate band); DORB ₹13,000.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="29" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>• Groundnut kernel ₹90,000 (Madurai mandi pod ₹6,500/qtl → kernel); Filtered groundnut oil ₹175,000;</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="29" t="inlineStr">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  groundnut cake/DOC ₹27,000 (40-50% protein, IndiaMART Gujarat/TN).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="29" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>• Copra (milling) ₹120,000 — near MSP ₹11,582/qtl (2025 season); Pollachi mandi range ₹4,700-15,349;</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="29" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  Coconut oil ₹250,000 (Indian premium; global $2,197-2,836/t, India premium 2x); coconut cake ₹35,000.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="29" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>• Oil yields: RBO 16-18% of bran; groundnut 42-48% of kernel; coconut 60-68% of copra (≈63% used).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="29" t="inlineStr"/>
+      <c r="B12" s="31" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="B13" s="29" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>WHY A COMBINED MILL (TN logic)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="29" t="inlineStr">
+      <c r="B14" s="31" t="inlineStr">
         <is>
           <t>• Coimbatore-Dindigul-Pollachi is India's edible-oil milling belt — copra + groundnut are TN's own crops,</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="29" t="inlineStr">
+      <c r="B15" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  rice bran comes captive from the paddy mill (Cauvery delta). One solvent-extraction + refinery line and</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="29" t="inlineStr">
+      <c r="B16" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  a husk-fired boiler serve all three → shared capex, diversified feedstock-price risk.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="29" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>• Coconut is the earner; RBO the steady base; groundnut the strategic/traditional line.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="29" t="inlineStr"/>
+      <c r="B18" s="31" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="B19" s="29" t="inlineStr">
+      <c r="B19" s="31" t="inlineStr">
         <is>
           <t>SEA (Solvent Extractors' Association of India)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="31" t="inlineStr">
         <is>
           <t>• seaofindia.com publishes daily oil rates, oilmeal export data, and crop estimates — the industry price</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="29" t="inlineStr">
+      <c r="B21" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  reference. ~350 member plants, ~30 MT crush capacity. Use SEA daily rates to refresh the oil-price inputs.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="29" t="inlineStr"/>
+      <c r="B22" s="31" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="B23" s="29" t="inlineStr">
+      <c r="B23" s="31" t="inlineStr">
         <is>
           <t>RETURNS (honest)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B24" s="31" t="inlineStr">
         <is>
           <t>• Combined EBITDA ~12%, PAT ~6%, Project IRR ~37% — but coconut-price-driven and</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="29" t="inlineStr">
+      <c r="B25" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">  volatile (see sensitivity). Groundnut line is loss-making at current prices; coconut + shared infra carry it.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="29" t="inlineStr">
+      <c r="B26" s="31" t="inlineStr">
         <is>
           <t>• Attractive but NOT low-risk: copra/coconut price swings are the dominant variable. Size debt against ₹225/kg.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="29" t="inlineStr"/>
+      <c r="B27" s="31" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="B28" s="29" t="inlineStr">
+      <c r="B28" s="31" t="inlineStr">
         <is>
           <t>SOURCES: SEA (seaofindia.com); copra MSP PIB PRID 2086629; Pollachi/TN copra &amp; coconut-oil-cake (commodityonline,</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="29" t="inlineStr">
+      <c r="B29" s="31" t="inlineStr">
         <is>
           <t>IndiaMART Coimbatore); groundnut (Agmarknet Madurai + IndiaMART); RBO/DORB (Business Standard, IndiaMART);</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="29" t="inlineStr">
+      <c r="B30" s="31" t="inlineStr">
         <is>
           <t>coconut oil global (AgroReview/Statista Q1-2026). Illustrative — a bankable DPR needs firm machinery quotes. Not investment advice.</t>
         </is>

</xml_diff>

<commit_message>
model: add Fuel Choice (husk/CBG Rs1/kWh vs grid Rs10.45/diesel Rs28 = Rs2.7-7.9cr/yr lever) + CBG Loop & Doubling Farmers' Income sheets to oil mill
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pitch/TN-Combined-Oil-Mill-Model.xlsx
+++ b/pitch/TN-Combined-Oil-Mill-Model.xlsx
@@ -13,6 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coconut-Price Sensitivity" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fodder (Oil-Cake) Margin" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SEA Prices &amp; Sources" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuel Choice — Mill Savings" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CBG Loop &amp; Doubling Income" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,12 +23,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="+#,##0.00;-#,##0.00"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,6 +97,15 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00b7791f"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
+      <sz val="9.5"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -125,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,6 +170,13 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1846,4 +1865,514 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Fuel choice for the mill — the hidden margin lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>The mill's energy can cost ₹0.5 or ₹28 per kWh depending on fuel. Captive husk/CBG vs grid/diesel = ₹2.7-7.9 cr/yr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>MILL ENERGY NEED</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Feedstock processed / yr (t)</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>11500</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Energy intensity (kWh-eq/t, steam+power)</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>solvent extraction + refining</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Total energy need (M kWh/yr)</t>
+        </is>
+      </c>
+      <c r="C8" s="32" t="n">
+        <v>2.88</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>FUEL OPTIONS — cost of the same 2.88 M kWh</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="4" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Fuel choice</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>₹/kWh</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>₹ cr/yr</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>vs husk</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>CBG (own de-oiled cake/residue)</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D12" s="33" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E12" s="34" t="n">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Rice husk boiler (captive)</t>
+        </is>
+      </c>
+      <c r="C13" s="32" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D13" s="33" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E13" s="34" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Solar (captive rooftop)</t>
+        </is>
+      </c>
+      <c r="C14" s="32" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="D14" s="35" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="E14" s="34" t="n">
+        <v>0.73</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Grid power (TANGEDCO HT)</t>
+        </is>
+      </c>
+      <c r="C15" s="32" t="n">
+        <v>10.45</v>
+      </c>
+      <c r="D15" s="36" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="34" t="n">
+        <v>2.72</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Diesel genset</t>
+        </is>
+      </c>
+      <c r="C16" s="32" t="n">
+        <v>28.47</v>
+      </c>
+      <c r="D16" s="36" t="n">
+        <v>8.19</v>
+      </c>
+      <c r="E16" s="34" t="n">
+        <v>7.909999999999999</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>→ Husk-fired boiler (₹0.99/kWh) vs GRID (₹10.45) saves ₹2.7 cr/yr; vs DIESEL genset saves ₹7.9 cr/yr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>→ On the mill's ₹12.3 cr EBITDA, the fuel choice is one of the BIGGEST single margin levers —</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  bigger than the groundnut line's whole contribution. Choosing captive husk/CBG is decisive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="37" t="inlineStr">
+        <is>
+          <t>→ CBG from the mill's OWN de-oiled cake + coconut shell/husk is cheaper still (₹0.45/kWh) and</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  makes the mill energy-self-sufficient — the same residue-to-energy loop as the farm side.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="37" t="inlineStr">
+        <is>
+          <t>→ WHY IT MATTERS: this is why oil mills co-locate with rice mills (husk) in the TN oil belt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A diesel/grid-run mill would lose most of its margin to energy; a husk/CBG mill keeps it.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2.5" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="B2" s="1" t="inlineStr">
+        <is>
+          <t>Farmer side — CBG loop &amp; Doubling Farmers' Income (DFI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>How the oil mill + CBG loop raises the groundnut/coconut farmer's income — the supply-side of the mill.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>CBG LOOP — farmer cost of production (groundnut, per ha)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="n"/>
+      <c r="D5" s="4" t="n"/>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5" s="4" t="n"/>
+      <c r="H5" s="4" t="n"/>
+    </row>
+    <row r="6">
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CNG fuel saving vs diesel (tractor)</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>3600</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>24% on fuel; ₹/ha</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Net residue income (haulm/shell → CBG/feed)</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>groundnut haulm + shell</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Net FOM (break-even yr1)</t>
+        </is>
+      </c>
+      <c r="C8" s="29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>soil-health positive long-term</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9">
+        <f> CBG loop benefit / ha</f>
+        <v/>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>6100</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>~6-8% of groundnut A2+FL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>DOUBLING FARMERS' INCOME — the mill's 4 contributions</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="4" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="4" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1. Real prices — assured local processing offtake</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>~5-8% farmgate uplift on oilseed/copra</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2. Cost saving — CBG loop (fuel+residue)</t>
+        </is>
+      </c>
+      <c r="C13" s="29" t="n">
+        <v>6100</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>₹/ha (above)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3. Byproduct income — shell/husk/haulm→CBG+feed</t>
+        </is>
+      </c>
+      <c r="C14" s="29" t="n">
+        <v>2500</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>resource-efficiency lever</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>4. Non-farm income — FPO share of mill PAT</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>₹7 cr PAT shared if farmer/FPO-owned</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="37" t="inlineStr">
+        <is>
+          <t>→ The Doubling Farmers' Income framework (Dalwai Committee) names 7 income sources. The combined</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  oil mill + CBG loop hits FOUR of them at once: real prices, cost reduction, resource efficiency,</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  and non-farm (processing) income — the same crop, four income streams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>→ A farmer supplying the mill AND running the CBG loop AND holding an FPO share captures:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  higher farmgate price + lower cost of production + residue income + a slice of the processing margin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="37" t="inlineStr">
+        <is>
+          <t>→ The mill does not double income alone — but it is exactly the 'value-addition + real-price + cost-cut'</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  combination the DFI strategy calls for, anchored in TN's own crops (groundnut, coconut, paddy-bran).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="37" t="inlineStr">
+        <is>
+          <t>→ THE FULL LOOP: crop → oil mill (price+jobs) → cake to Namakkal poultry (feed) → husk/CBG fuels the</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  mill AND the farmer's tractor → slurry to the field. Every residue becomes income or energy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Sources: Dalwai Committee (Doubling Farmers' Income, 2018, 7 sources); CACP A2+FL; PIB CNG-tractor &amp; SATAT CBG;</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>TN diesel/CNG Jul 2026; this workbook's mill P&amp;L. Illustrative — the DFI uplift is directional, not a guarantee.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>